<commit_message>
Big updates - testing logic (broken interface) and first basic testing tests
</commit_message>
<xml_diff>
--- a/data/tier_app/tier_app_params.xlsx
+++ b/data/tier_app/tier_app_params.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/tier_app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="528" documentId="8_{3983ECF5-E0D1-344B-BC04-D4E6CF5CD4B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D386A8D2-4993-0649-9C64-561A1E0CEB5F}"/>
+  <xr:revisionPtr revIDLastSave="531" documentId="8_{3983ECF5-E0D1-344B-BC04-D4E6CF5CD4B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D14EEC3-3143-8A41-A247-992F22562BDD}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="540" windowWidth="28800" windowHeight="16020" activeTab="1" xr2:uid="{BFD43C4F-988C-0F4F-AE69-989101776492}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" activeTab="2" xr2:uid="{BFD43C4F-988C-0F4F-AE69-989101776492}"/>
   </bookViews>
   <sheets>
     <sheet name="param_list_and_type" sheetId="2" r:id="rId1"/>
     <sheet name="tier_plus_updated" sheetId="6" r:id="rId2"/>
-    <sheet name="baseline_data" sheetId="4" r:id="rId3"/>
-    <sheet name="params_effect" sheetId="1" r:id="rId4"/>
-    <sheet name="other_key_values" sheetId="5" r:id="rId5"/>
-    <sheet name="params_cost" sheetId="3" r:id="rId6"/>
+    <sheet name="tier_plus_30Jan" sheetId="7" r:id="rId3"/>
+    <sheet name="baseline_data" sheetId="4" r:id="rId4"/>
+    <sheet name="params_effect" sheetId="1" r:id="rId5"/>
+    <sheet name="other_key_values" sheetId="5" r:id="rId6"/>
+    <sheet name="params_cost" sheetId="3" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">params_effect!$A$1:$L$205</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">params_effect!$A$1:$L$205</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -66,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1625" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1838" uniqueCount="204">
   <si>
     <t>area</t>
   </si>
@@ -626,6 +627,60 @@
   </si>
   <si>
     <t>https://bushare-my.sharepoint.com/:x:/g/personal/brooken_bu_edu/IQCrAqcnpglYQbFHxzN39mrIAddSipC0bePCNG6CgXoCMBk?e=5xvACO</t>
+  </si>
+  <si>
+    <t>Cotrimoxazole prophylaxis (according to guidelines)</t>
+  </si>
+  <si>
+    <t>tb_test_treat</t>
+  </si>
+  <si>
+    <t>TB Screening and Treatment</t>
+  </si>
+  <si>
+    <t>tpt</t>
+  </si>
+  <si>
+    <t>TPT provision</t>
+  </si>
+  <si>
+    <t>AHD testing and prophylaxis package (LAM, CrAG, CD4, fluconazole)</t>
+  </si>
+  <si>
+    <t>cags</t>
+  </si>
+  <si>
+    <t>Community ART Groups</t>
+  </si>
+  <si>
+    <t>Testing: facility-based (general)</t>
+  </si>
+  <si>
+    <t>Testing: facility-based (targeted)</t>
+  </si>
+  <si>
+    <t>Testing: Network/Index</t>
+  </si>
+  <si>
+    <t>PNC</t>
+  </si>
+  <si>
+    <t>pnc_hiv_test</t>
+  </si>
+  <si>
+    <t>PNC: HIV testing</t>
+  </si>
+  <si>
+    <t>pnc_vl_testing</t>
+  </si>
+  <si>
+    <t>PNC: Viral Load Testing</t>
+  </si>
+  <si>
+    <t>pnc_art_cont</t>
+  </si>
+  <si>
+    <t>PNC: ART continuation</t>
   </si>
 </sst>
 </file>
@@ -733,7 +788,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -773,6 +828,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2841,6 +2899,874 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4335FE8B-B359-CC48-8F11-F322EA2E822B}">
+  <dimension ref="A1:K33"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:11" ht="238" x14ac:dyDescent="0.2">
+      <c r="A1" s="17"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="20" t="s">
+        <v>167</v>
+      </c>
+      <c r="F1" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>169</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="G2" s="18" t="s">
+        <v>171</v>
+      </c>
+      <c r="H2" s="18" t="s">
+        <v>172</v>
+      </c>
+      <c r="I2" s="18" t="s">
+        <v>173</v>
+      </c>
+      <c r="J2" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="K2" s="18" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="J3" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="K3" s="17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="K4" s="17"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="17"/>
+      <c r="K5" s="17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="K6" s="17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="K7" s="17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="K8" s="17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="17"/>
+      <c r="K10" s="17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="17"/>
+      <c r="K11" s="17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="J12" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="K12" s="17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="J13" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="K13" s="17"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="J14" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="K14" s="17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="I15" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="J15" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="K15" s="17"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="I16" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="J16" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="K16" s="17"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A17" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="I17" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="J17" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="K17" s="17"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A18" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="I18" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="J18" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="K18" s="17"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A19" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="I19" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="J19" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="K19" s="17"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A20" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="I20" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="J20" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="K20" s="17"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A21" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="I21" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="J21" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="K21" s="17"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A22" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F22" s="17"/>
+      <c r="G22" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H22" s="17"/>
+      <c r="I22" s="17"/>
+      <c r="J22" s="17"/>
+      <c r="K22" s="17"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A23" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G23" s="17"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="17"/>
+      <c r="J23" s="17"/>
+      <c r="K23" s="17"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A24" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F24" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
+      <c r="J24" s="17"/>
+      <c r="K24" s="17"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A25" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F25" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="17"/>
+      <c r="K25" s="17"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A26" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F26" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="G26" s="17"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="17"/>
+      <c r="J26" s="17"/>
+      <c r="K26" s="17"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A27" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F27" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="G27" s="17"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="17"/>
+      <c r="K27" s="17"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A28" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F28" s="17"/>
+      <c r="G28" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H28" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="I28" s="17"/>
+      <c r="J28" s="17"/>
+      <c r="K28" s="17"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A29" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F29" s="17"/>
+      <c r="G29" s="17"/>
+      <c r="H29" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="I29" s="17"/>
+      <c r="J29" s="17"/>
+      <c r="K29" s="17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A30" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F30" s="17"/>
+      <c r="G30" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H30" s="17"/>
+      <c r="I30" s="17"/>
+      <c r="J30" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="K30" s="17"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A31" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F31" s="17"/>
+      <c r="G31" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H31" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="I31" s="17"/>
+      <c r="J31" s="17"/>
+      <c r="K31" s="17"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A32" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F32" s="17"/>
+      <c r="G32" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H32" s="17"/>
+      <c r="I32" s="17"/>
+      <c r="J32" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="K32" s="17"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A33" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="D33" s="17"/>
+      <c r="E33" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F33" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="G33" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H33" s="17"/>
+      <c r="I33" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="J33" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="K33" s="17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="F1:K1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBDA1724-5B29-934D-97A3-4F5620D9530D}">
   <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3032,7 +3958,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58B67A41-5C08-024B-8E12-B539DFD980B2}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:L205"/>
@@ -10452,7 +11378,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE40B620-F4DF-C944-9DE6-37E48F558719}">
   <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -10518,7 +11444,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7C1EB35-7EE8-BE4D-9B8E-69F9F2C4B9B0}">
   <dimension ref="A1:F206"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>